<commit_message>
SỬA LỖI: đổi simple average thành weighted average
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data\Code\Python\ML WS\challenge1_titanic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DC384FB-1135-4F18-98F7-CCE69DECAAED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A44E467-ED8C-4C71-9AD9-AFA9A38FB1CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19305" yWindow="240" windowWidth="9255" windowHeight="15270" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="01_feature_engineering" sheetId="1" r:id="rId1"/>
-    <sheet name="02_ensemble" sheetId="2" r:id="rId2"/>
+    <sheet name="Baseline" sheetId="3" r:id="rId1"/>
+    <sheet name="01_feature_engineering" sheetId="1" r:id="rId2"/>
+    <sheet name="02_ensemble" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="40">
   <si>
     <t>LR</t>
   </si>
@@ -82,9 +83,6 @@
     <t>Kaggle (Accuracy)</t>
   </si>
   <si>
-    <t>Baseline(SVM)</t>
-  </si>
-  <si>
     <t>Model</t>
   </si>
   <si>
@@ -112,13 +110,43 @@
     <t>Accuracy Score</t>
   </si>
   <si>
-    <t>Simple average (LDA, RF, LR)</t>
-  </si>
-  <si>
     <t>Voting (LDA, RF)</t>
   </si>
   <si>
     <t>Stacking (LDA, RF, LR + LogisticRegression)</t>
+  </si>
+  <si>
+    <t>0.805825 +/- 0.025845</t>
+  </si>
+  <si>
+    <t>0.802486 +/- 0.032724</t>
+  </si>
+  <si>
+    <t>0.726144 +/- 0.017993</t>
+  </si>
+  <si>
+    <t>0.782286 +/- 0.019678</t>
+  </si>
+  <si>
+    <t>0.776656 +/- 0.020832</t>
+  </si>
+  <si>
+    <t>CART</t>
+  </si>
+  <si>
+    <t>NB</t>
+  </si>
+  <si>
+    <t>Tunning</t>
+  </si>
+  <si>
+    <t>Best param</t>
+  </si>
+  <si>
+    <t>{'n_neighbors': 6}</t>
+  </si>
+  <si>
+    <t>Weighted average (LDA, RF, LR)</t>
   </si>
 </sst>
 </file>
@@ -442,6 +470,110 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CE11E13-E6EE-45C3-BCB6-F9F03104C730}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="28.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="60.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0.71938359173937605</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.78674910551754396</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.76793999999999996</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -457,10 +589,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>11</v>
@@ -472,7 +604,7 @@
         <v>17</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -509,7 +641,7 @@
         <v>0.77510999999999997</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -529,7 +661,7 @@
         <v>0.67942999999999998</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -566,25 +698,11 @@
         <v>0.77032999999999996</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="1">
-        <v>0.78674910551754396</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="1">
-        <v>0.76793999999999996</v>
-      </c>
+      <c r="B7" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -592,7 +710,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7407A8A-5BC5-4CAF-8421-FD26C2DB8B05}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -604,10 +722,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>17</v>
@@ -615,7 +733,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B2" s="1">
         <v>0.83052700000000002</v>
@@ -626,7 +744,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B3" s="1">
         <v>0.83277199999999996</v>
@@ -637,7 +755,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B4" s="1">
         <v>0.82122899999999999</v>

</xml_diff>